<commit_message>
feat (hash) : ajouté le hashage des mdp + sel
</commit_message>
<xml_diff>
--- a/Journal-de-Travail_BorminKiril.xlsx
+++ b/Journal-de-Travail_BorminKiril.xlsx
@@ -5,12 +5,12 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\px20umf\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\px20umf\Documents\GitHub\secured_webshop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BFCB1FA0-D805-4532-A983-DAC096BE3EEE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A9A303B0-29BD-4CBE-88CF-394C93E6E30E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5280" yWindow="2325" windowWidth="21600" windowHeight="11385" xr2:uid="{6CC57B32-2488-5244-B7A6-FB7E808234AC}"/>
+    <workbookView xWindow="5625" yWindow="2670" windowWidth="21600" windowHeight="11385" xr2:uid="{6CC57B32-2488-5244-B7A6-FB7E808234AC}"/>
   </bookViews>
   <sheets>
     <sheet name="Journal de travail" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="37">
   <si>
     <t>Journal de travail</t>
   </si>
@@ -149,6 +149,9 @@
   </si>
   <si>
     <t xml:space="preserve">Créer la page d'inscription </t>
+  </si>
+  <si>
+    <t>Ajout de hachage de mpd + sel</t>
   </si>
 </sst>
 </file>
@@ -1159,7 +1162,7 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>120</c:v>
+                  <c:v>160</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>0</c:v>
@@ -4255,7 +4258,7 @@
       <c r="B3" s="86"/>
       <c r="C3" s="67" t="str">
         <f>QUOTIENT(E4,60)&amp;" heures "&amp;MOD(E4,60)&amp;" minutes"</f>
-        <v>2 heures 0 minutes</v>
+        <v>2 heures 40 minutes</v>
       </c>
       <c r="D3" s="17"/>
       <c r="E3" s="3"/>
@@ -4274,11 +4277,11 @@
       </c>
       <c r="D4" s="17">
         <f>SUBTOTAL(9,$D$7:$D$531)</f>
-        <v>60</v>
+        <v>100</v>
       </c>
       <c r="E4" s="24">
         <f>SUM(C4:D4)</f>
-        <v>120</v>
+        <v>160</v>
       </c>
       <c r="F4" s="4"/>
       <c r="G4" s="6"/>
@@ -4393,15 +4396,23 @@
       </c>
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A10" s="62" t="str">
+      <c r="A10" s="62">
         <f>IF(ISBLANK(B10),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B10))</f>
-        <v/>
-      </c>
-      <c r="B10" s="30"/>
+        <v>13</v>
+      </c>
+      <c r="B10" s="30">
+        <v>46108</v>
+      </c>
       <c r="C10" s="31"/>
-      <c r="D10" s="32"/>
-      <c r="E10" s="33"/>
-      <c r="F10" s="23"/>
+      <c r="D10" s="32">
+        <v>40</v>
+      </c>
+      <c r="E10" s="33" t="s">
+        <v>15</v>
+      </c>
+      <c r="F10" s="23" t="s">
+        <v>36</v>
+      </c>
       <c r="G10" s="39"/>
       <c r="M10" t="s">
         <v>16</v>
@@ -10900,11 +10911,11 @@
       </c>
       <c r="B7">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Plannification!E7,'Journal de travail'!$D$7:$D$532)</f>
-        <v>60</v>
+        <v>100</v>
       </c>
       <c r="C7">
         <f t="shared" si="0"/>
-        <v>120</v>
+        <v>160</v>
       </c>
       <c r="E7" s="73" t="str">
         <f>'Journal de travail'!M9</f>
@@ -10912,7 +10923,7 @@
       </c>
       <c r="F7" s="74" t="str">
         <f t="shared" ref="F7:F11" si="1">QUOTIENT(SUM(A7:B7),60)&amp;" h "&amp;TEXT(MOD(SUM(A7:B7),60), "00")&amp;" min"</f>
-        <v>2 h 00 min</v>
+        <v>2 h 40 min</v>
       </c>
       <c r="G7" s="75">
         <f t="shared" ref="G7:G9" si="2">SUM(A7:B7)/$C$11</f>
@@ -11046,22 +11057,22 @@
       </c>
       <c r="B11">
         <f>SUM(B6:B10)</f>
-        <v>60</v>
+        <v>100</v>
       </c>
       <c r="C11">
         <f>SUM(A11:B11)</f>
-        <v>120</v>
+        <v>160</v>
       </c>
       <c r="E11" s="81" t="s">
         <v>29</v>
       </c>
       <c r="F11" s="71" t="str">
         <f t="shared" si="1"/>
-        <v>2 h 00 min</v>
+        <v>2 h 40 min</v>
       </c>
       <c r="G11" s="82">
         <f>C11/C12</f>
-        <v>2.2222222222222223E-2</v>
+        <v>2.9629629629629631E-2</v>
       </c>
       <c r="L11" s="56" t="s">
         <v>29</v>
@@ -11100,6 +11111,26 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="f20a0681-8b2f-4a46-9dab-cf1520193f81">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="932fafb7-d8e0-4a14-bee3-33aad5c71309" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101005B1120F001D1794FAA6F4057E3355991" ma:contentTypeVersion="10" ma:contentTypeDescription="Crée un document." ma:contentTypeScope="" ma:versionID="62349bcdb43c26c508700efba1cb50b1">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="f20a0681-8b2f-4a46-9dab-cf1520193f81" xmlns:ns3="932fafb7-d8e0-4a14-bee3-33aad5c71309" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="0e5d6db3f342a25e0e30f4a2965162e1" ns2:_="" ns3:_="">
     <xsd:import namespace="f20a0681-8b2f-4a46-9dab-cf1520193f81"/>
@@ -11288,27 +11319,32 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0453EC0E-0298-408B-815C-A1500DB4F5E9}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="932fafb7-d8e0-4a14-bee3-33aad5c71309"/>
+    <ds:schemaRef ds:uri="f20a0681-8b2f-4a46-9dab-cf1520193f81"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="f20a0681-8b2f-4a46-9dab-cf1520193f81">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="932fafb7-d8e0-4a14-bee3-33aad5c71309" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{74326215-CB02-4E95-BFFB-9EC625B1BF0F}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1424D28F-D6A9-45ED-AED5-A0D744400EE5}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -11325,29 +11361,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{74326215-CB02-4E95-BFFB-9EC625B1BF0F}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0453EC0E-0298-408B-815C-A1500DB4F5E9}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="932fafb7-d8e0-4a14-bee3-33aad5c71309"/>
-    <ds:schemaRef ds:uri="f20a0681-8b2f-4a46-9dab-cf1520193f81"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
feat (jwt) : générer jwt token pour les users WIP
</commit_message>
<xml_diff>
--- a/Journal-de-Travail_BorminKiril.xlsx
+++ b/Journal-de-Travail_BorminKiril.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\px20umf\Documents\GitHub\secured_webshop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A9A303B0-29BD-4CBE-88CF-394C93E6E30E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{67C824DB-C7E6-4356-A8E5-D8D7ECCA7781}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="5625" yWindow="2670" windowWidth="21600" windowHeight="11385" xr2:uid="{6CC57B32-2488-5244-B7A6-FB7E808234AC}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="38">
   <si>
     <t>Journal de travail</t>
   </si>
@@ -152,6 +152,9 @@
   </si>
   <si>
     <t>Ajout de hachage de mpd + sel</t>
+  </si>
+  <si>
+    <t>Ajout de poivre</t>
   </si>
 </sst>
 </file>
@@ -1162,7 +1165,7 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>160</c:v>
+                  <c:v>180</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>0</c:v>
@@ -4258,7 +4261,7 @@
       <c r="B3" s="86"/>
       <c r="C3" s="67" t="str">
         <f>QUOTIENT(E4,60)&amp;" heures "&amp;MOD(E4,60)&amp;" minutes"</f>
-        <v>2 heures 40 minutes</v>
+        <v>3 heures 0 minutes</v>
       </c>
       <c r="D3" s="17"/>
       <c r="E3" s="3"/>
@@ -4277,11 +4280,11 @@
       </c>
       <c r="D4" s="17">
         <f>SUBTOTAL(9,$D$7:$D$531)</f>
-        <v>100</v>
+        <v>120</v>
       </c>
       <c r="E4" s="24">
         <f>SUM(C4:D4)</f>
-        <v>160</v>
+        <v>180</v>
       </c>
       <c r="F4" s="4"/>
       <c r="G4" s="6"/>
@@ -4425,15 +4428,23 @@
       </c>
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A11" s="63" t="str">
+      <c r="A11" s="63">
         <f>IF(ISBLANK(B11),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B11))</f>
-        <v/>
-      </c>
-      <c r="B11" s="34"/>
+        <v>13</v>
+      </c>
+      <c r="B11" s="34">
+        <v>46108</v>
+      </c>
       <c r="C11" s="35"/>
-      <c r="D11" s="36"/>
-      <c r="E11" s="37"/>
-      <c r="F11" s="23"/>
+      <c r="D11" s="36">
+        <v>20</v>
+      </c>
+      <c r="E11" s="37" t="s">
+        <v>15</v>
+      </c>
+      <c r="F11" s="23" t="s">
+        <v>37</v>
+      </c>
       <c r="G11" s="40"/>
       <c r="M11" t="s">
         <v>17</v>
@@ -10911,11 +10922,11 @@
       </c>
       <c r="B7">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Plannification!E7,'Journal de travail'!$D$7:$D$532)</f>
-        <v>100</v>
+        <v>120</v>
       </c>
       <c r="C7">
         <f t="shared" si="0"/>
-        <v>160</v>
+        <v>180</v>
       </c>
       <c r="E7" s="73" t="str">
         <f>'Journal de travail'!M9</f>
@@ -10923,7 +10934,7 @@
       </c>
       <c r="F7" s="74" t="str">
         <f t="shared" ref="F7:F11" si="1">QUOTIENT(SUM(A7:B7),60)&amp;" h "&amp;TEXT(MOD(SUM(A7:B7),60), "00")&amp;" min"</f>
-        <v>2 h 40 min</v>
+        <v>3 h 00 min</v>
       </c>
       <c r="G7" s="75">
         <f t="shared" ref="G7:G9" si="2">SUM(A7:B7)/$C$11</f>
@@ -11057,22 +11068,22 @@
       </c>
       <c r="B11">
         <f>SUM(B6:B10)</f>
-        <v>100</v>
+        <v>120</v>
       </c>
       <c r="C11">
         <f>SUM(A11:B11)</f>
-        <v>160</v>
+        <v>180</v>
       </c>
       <c r="E11" s="81" t="s">
         <v>29</v>
       </c>
       <c r="F11" s="71" t="str">
         <f t="shared" si="1"/>
-        <v>2 h 40 min</v>
+        <v>3 h 00 min</v>
       </c>
       <c r="G11" s="82">
         <f>C11/C12</f>
-        <v>2.9629629629629631E-2</v>
+        <v>3.3333333333333333E-2</v>
       </c>
       <c r="L11" s="56" t="s">
         <v>29</v>
@@ -11111,6 +11122,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="f20a0681-8b2f-4a46-9dab-cf1520193f81">
@@ -11119,15 +11139,6 @@
     <TaxCatchAll xmlns="932fafb7-d8e0-4a14-bee3-33aad5c71309" xsi:nil="true"/>
   </documentManagement>
 </p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -11320,6 +11331,14 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{74326215-CB02-4E95-BFFB-9EC625B1BF0F}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0453EC0E-0298-408B-815C-A1500DB4F5E9}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
@@ -11332,14 +11351,6 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
     <ds:schemaRef ds:uri="932fafb7-d8e0-4a14-bee3-33aad5c71309"/>
     <ds:schemaRef ds:uri="f20a0681-8b2f-4a46-9dab-cf1520193f81"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{74326215-CB02-4E95-BFFB-9EC625B1BF0F}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>

<commit_message>
chore (.env) : suppression de la variable d'environnement du repo git
</commit_message>
<xml_diff>
--- a/Journal-de-Travail_BorminKiril.xlsx
+++ b/Journal-de-Travail_BorminKiril.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\px20umf\Documents\GitHub\secured_webshop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{67C824DB-C7E6-4356-A8E5-D8D7ECCA7781}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D1E2827-9D6C-4EB0-AFBD-5E10CECDD683}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="5625" yWindow="2670" windowWidth="21600" windowHeight="11385" xr2:uid="{6CC57B32-2488-5244-B7A6-FB7E808234AC}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="39">
   <si>
     <t>Journal de travail</t>
   </si>
@@ -155,6 +155,9 @@
   </si>
   <si>
     <t>Ajout de poivre</t>
+  </si>
+  <si>
+    <t>Ajout de token jwt WIP</t>
   </si>
 </sst>
 </file>
@@ -1165,7 +1168,7 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>180</c:v>
+                  <c:v>195</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>0</c:v>
@@ -4261,7 +4264,7 @@
       <c r="B3" s="86"/>
       <c r="C3" s="67" t="str">
         <f>QUOTIENT(E4,60)&amp;" heures "&amp;MOD(E4,60)&amp;" minutes"</f>
-        <v>3 heures 0 minutes</v>
+        <v>3 heures 15 minutes</v>
       </c>
       <c r="D3" s="17"/>
       <c r="E3" s="3"/>
@@ -4280,11 +4283,11 @@
       </c>
       <c r="D4" s="17">
         <f>SUBTOTAL(9,$D$7:$D$531)</f>
-        <v>120</v>
+        <v>135</v>
       </c>
       <c r="E4" s="24">
         <f>SUM(C4:D4)</f>
-        <v>180</v>
+        <v>195</v>
       </c>
       <c r="F4" s="4"/>
       <c r="G4" s="6"/>
@@ -4457,15 +4460,23 @@
       </c>
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A12" s="62" t="str">
+      <c r="A12" s="62">
         <f>IF(ISBLANK(B12),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B12))</f>
-        <v/>
-      </c>
-      <c r="B12" s="30"/>
+        <v>13</v>
+      </c>
+      <c r="B12" s="30">
+        <v>46108</v>
+      </c>
       <c r="C12" s="31"/>
-      <c r="D12" s="32"/>
-      <c r="E12" s="33"/>
-      <c r="F12" s="23"/>
+      <c r="D12" s="32">
+        <v>15</v>
+      </c>
+      <c r="E12" s="33" t="s">
+        <v>15</v>
+      </c>
+      <c r="F12" s="23" t="s">
+        <v>38</v>
+      </c>
       <c r="G12" s="39"/>
       <c r="M12" t="s">
         <v>18</v>
@@ -10922,11 +10933,11 @@
       </c>
       <c r="B7">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Plannification!E7,'Journal de travail'!$D$7:$D$532)</f>
-        <v>120</v>
+        <v>135</v>
       </c>
       <c r="C7">
         <f t="shared" si="0"/>
-        <v>180</v>
+        <v>195</v>
       </c>
       <c r="E7" s="73" t="str">
         <f>'Journal de travail'!M9</f>
@@ -10934,7 +10945,7 @@
       </c>
       <c r="F7" s="74" t="str">
         <f t="shared" ref="F7:F11" si="1">QUOTIENT(SUM(A7:B7),60)&amp;" h "&amp;TEXT(MOD(SUM(A7:B7),60), "00")&amp;" min"</f>
-        <v>3 h 00 min</v>
+        <v>3 h 15 min</v>
       </c>
       <c r="G7" s="75">
         <f t="shared" ref="G7:G9" si="2">SUM(A7:B7)/$C$11</f>
@@ -11068,22 +11079,22 @@
       </c>
       <c r="B11">
         <f>SUM(B6:B10)</f>
-        <v>120</v>
+        <v>135</v>
       </c>
       <c r="C11">
         <f>SUM(A11:B11)</f>
-        <v>180</v>
+        <v>195</v>
       </c>
       <c r="E11" s="81" t="s">
         <v>29</v>
       </c>
       <c r="F11" s="71" t="str">
         <f t="shared" si="1"/>
-        <v>3 h 00 min</v>
+        <v>3 h 15 min</v>
       </c>
       <c r="G11" s="82">
         <f>C11/C12</f>
-        <v>3.3333333333333333E-2</v>
+        <v>3.6111111111111108E-2</v>
       </c>
       <c r="L11" s="56" t="s">
         <v>29</v>
@@ -11122,15 +11133,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="f20a0681-8b2f-4a46-9dab-cf1520193f81">
@@ -11139,6 +11141,15 @@
     <TaxCatchAll xmlns="932fafb7-d8e0-4a14-bee3-33aad5c71309" xsi:nil="true"/>
   </documentManagement>
 </p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -11331,14 +11342,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{74326215-CB02-4E95-BFFB-9EC625B1BF0F}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0453EC0E-0298-408B-815C-A1500DB4F5E9}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
@@ -11351,6 +11354,14 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
     <ds:schemaRef ds:uri="932fafb7-d8e0-4a14-bee3-33aad5c71309"/>
     <ds:schemaRef ds:uri="f20a0681-8b2f-4a46-9dab-cf1520193f81"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{74326215-CB02-4E95-BFFB-9EC625B1BF0F}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>

<commit_message>
feat (routes) : vérification du token JWT
</commit_message>
<xml_diff>
--- a/Journal-de-Travail_BorminKiril.xlsx
+++ b/Journal-de-Travail_BorminKiril.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\px20umf\Documents\GitHub\secured_webshop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D1E2827-9D6C-4EB0-AFBD-5E10CECDD683}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{88849D4B-A891-44DB-B867-640189E79275}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="5625" yWindow="2670" windowWidth="21600" windowHeight="11385" xr2:uid="{6CC57B32-2488-5244-B7A6-FB7E808234AC}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="41">
   <si>
     <t>Journal de travail</t>
   </si>
@@ -158,6 +158,12 @@
   </si>
   <si>
     <t>Ajout de token jwt WIP</t>
+  </si>
+  <si>
+    <t>Finission d'ajout token jwt</t>
+  </si>
+  <si>
+    <t>Réaliser la protection de la page admin et ajout de rôles user et admin dans la bdd</t>
   </si>
 </sst>
 </file>
@@ -1168,7 +1174,7 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>195</c:v>
+                  <c:v>265</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>0</c:v>
@@ -4264,7 +4270,7 @@
       <c r="B3" s="86"/>
       <c r="C3" s="67" t="str">
         <f>QUOTIENT(E4,60)&amp;" heures "&amp;MOD(E4,60)&amp;" minutes"</f>
-        <v>3 heures 15 minutes</v>
+        <v>4 heures 25 minutes</v>
       </c>
       <c r="D3" s="17"/>
       <c r="E3" s="3"/>
@@ -4283,11 +4289,11 @@
       </c>
       <c r="D4" s="17">
         <f>SUBTOTAL(9,$D$7:$D$531)</f>
-        <v>135</v>
+        <v>205</v>
       </c>
       <c r="E4" s="24">
         <f>SUM(C4:D4)</f>
-        <v>195</v>
+        <v>265</v>
       </c>
       <c r="F4" s="4"/>
       <c r="G4" s="6"/>
@@ -4489,15 +4495,23 @@
       </c>
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A13" s="63" t="str">
+      <c r="A13" s="63">
         <f>IF(ISBLANK(B13),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B13))</f>
-        <v/>
-      </c>
-      <c r="B13" s="34"/>
+        <v>17</v>
+      </c>
+      <c r="B13" s="34">
+        <v>46136</v>
+      </c>
       <c r="C13" s="35"/>
-      <c r="D13" s="36"/>
-      <c r="E13" s="37"/>
-      <c r="F13" s="23"/>
+      <c r="D13" s="36">
+        <v>30</v>
+      </c>
+      <c r="E13" s="37" t="s">
+        <v>15</v>
+      </c>
+      <c r="F13" s="23" t="s">
+        <v>39</v>
+      </c>
       <c r="G13" s="40"/>
       <c r="N13">
         <v>6</v>
@@ -4507,15 +4521,23 @@
       </c>
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A14" s="62" t="str">
+      <c r="A14" s="62">
         <f>IF(ISBLANK(B14),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B14))</f>
-        <v/>
-      </c>
-      <c r="B14" s="30"/>
+        <v>17</v>
+      </c>
+      <c r="B14" s="30">
+        <v>46136</v>
+      </c>
       <c r="C14" s="31"/>
-      <c r="D14" s="32"/>
-      <c r="E14" s="33"/>
-      <c r="F14" s="23"/>
+      <c r="D14" s="32">
+        <v>40</v>
+      </c>
+      <c r="E14" s="33" t="s">
+        <v>15</v>
+      </c>
+      <c r="F14" s="23" t="s">
+        <v>40</v>
+      </c>
       <c r="G14" s="39"/>
       <c r="N14">
         <v>7</v>
@@ -10933,11 +10955,11 @@
       </c>
       <c r="B7">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Plannification!E7,'Journal de travail'!$D$7:$D$532)</f>
-        <v>135</v>
+        <v>205</v>
       </c>
       <c r="C7">
         <f t="shared" si="0"/>
-        <v>195</v>
+        <v>265</v>
       </c>
       <c r="E7" s="73" t="str">
         <f>'Journal de travail'!M9</f>
@@ -10945,7 +10967,7 @@
       </c>
       <c r="F7" s="74" t="str">
         <f t="shared" ref="F7:F11" si="1">QUOTIENT(SUM(A7:B7),60)&amp;" h "&amp;TEXT(MOD(SUM(A7:B7),60), "00")&amp;" min"</f>
-        <v>3 h 15 min</v>
+        <v>4 h 25 min</v>
       </c>
       <c r="G7" s="75">
         <f t="shared" ref="G7:G9" si="2">SUM(A7:B7)/$C$11</f>
@@ -11079,22 +11101,22 @@
       </c>
       <c r="B11">
         <f>SUM(B6:B10)</f>
-        <v>135</v>
+        <v>205</v>
       </c>
       <c r="C11">
         <f>SUM(A11:B11)</f>
-        <v>195</v>
+        <v>265</v>
       </c>
       <c r="E11" s="81" t="s">
         <v>29</v>
       </c>
       <c r="F11" s="71" t="str">
         <f t="shared" si="1"/>
-        <v>3 h 15 min</v>
+        <v>4 h 25 min</v>
       </c>
       <c r="G11" s="82">
         <f>C11/C12</f>
-        <v>3.6111111111111108E-2</v>
+        <v>4.9074074074074076E-2</v>
       </c>
       <c r="L11" s="56" t="s">
         <v>29</v>
@@ -11133,6 +11155,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="f20a0681-8b2f-4a46-9dab-cf1520193f81">
@@ -11141,15 +11172,6 @@
     <TaxCatchAll xmlns="932fafb7-d8e0-4a14-bee3-33aad5c71309" xsi:nil="true"/>
   </documentManagement>
 </p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -11342,6 +11364,14 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{74326215-CB02-4E95-BFFB-9EC625B1BF0F}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0453EC0E-0298-408B-815C-A1500DB4F5E9}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
@@ -11354,14 +11384,6 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
     <ds:schemaRef ds:uri="932fafb7-d8e0-4a14-bee3-33aad5c71309"/>
     <ds:schemaRef ds:uri="f20a0681-8b2f-4a46-9dab-cf1520193f81"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{74326215-CB02-4E95-BFFB-9EC625B1BF0F}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>

<commit_message>
feat (mdp) : ajout d'une politique de mdp fort
</commit_message>
<xml_diff>
--- a/Journal-de-Travail_BorminKiril.xlsx
+++ b/Journal-de-Travail_BorminKiril.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\px20umf\Documents\GitHub\secured_webshop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{88849D4B-A891-44DB-B867-640189E79275}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{980013FA-AA14-4D33-A015-86C899159C3A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="5625" yWindow="2670" windowWidth="21600" windowHeight="11385" xr2:uid="{6CC57B32-2488-5244-B7A6-FB7E808234AC}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="43">
   <si>
     <t>Journal de travail</t>
   </si>
@@ -164,6 +164,12 @@
   </si>
   <si>
     <t>Réaliser la protection de la page admin et ajout de rôles user et admin dans la bdd</t>
+  </si>
+  <si>
+    <t>Réalisation de https</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ajout de politique de mdp </t>
   </si>
 </sst>
 </file>
@@ -1174,7 +1180,7 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>265</c:v>
+                  <c:v>315</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>0</c:v>
@@ -4270,7 +4276,7 @@
       <c r="B3" s="86"/>
       <c r="C3" s="67" t="str">
         <f>QUOTIENT(E4,60)&amp;" heures "&amp;MOD(E4,60)&amp;" minutes"</f>
-        <v>4 heures 25 minutes</v>
+        <v>5 heures 15 minutes</v>
       </c>
       <c r="D3" s="17"/>
       <c r="E3" s="3"/>
@@ -4289,11 +4295,11 @@
       </c>
       <c r="D4" s="17">
         <f>SUBTOTAL(9,$D$7:$D$531)</f>
-        <v>205</v>
+        <v>255</v>
       </c>
       <c r="E4" s="24">
         <f>SUM(C4:D4)</f>
-        <v>265</v>
+        <v>315</v>
       </c>
       <c r="F4" s="4"/>
       <c r="G4" s="6"/>
@@ -4504,7 +4510,7 @@
       </c>
       <c r="C13" s="35"/>
       <c r="D13" s="36">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="E13" s="37" t="s">
         <v>15</v>
@@ -4530,7 +4536,7 @@
       </c>
       <c r="C14" s="31"/>
       <c r="D14" s="32">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="E14" s="33" t="s">
         <v>15</v>
@@ -4547,15 +4553,23 @@
       </c>
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A15" s="63" t="str">
+      <c r="A15" s="63">
         <f>IF(ISBLANK(B15),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B15))</f>
-        <v/>
-      </c>
-      <c r="B15" s="34"/>
+        <v>17</v>
+      </c>
+      <c r="B15" s="34">
+        <v>46136</v>
+      </c>
       <c r="C15" s="35"/>
-      <c r="D15" s="36"/>
-      <c r="E15" s="37"/>
-      <c r="F15" s="23"/>
+      <c r="D15" s="36">
+        <v>40</v>
+      </c>
+      <c r="E15" s="37" t="s">
+        <v>15</v>
+      </c>
+      <c r="F15" s="23" t="s">
+        <v>41</v>
+      </c>
       <c r="G15" s="40"/>
       <c r="N15">
         <v>8</v>
@@ -4565,15 +4579,23 @@
       </c>
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A16" s="62" t="str">
+      <c r="A16" s="62">
         <f>IF(ISBLANK(B16),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B16))</f>
-        <v/>
-      </c>
-      <c r="B16" s="30"/>
+        <v>17</v>
+      </c>
+      <c r="B16" s="30">
+        <v>46136</v>
+      </c>
       <c r="C16" s="31"/>
-      <c r="D16" s="32"/>
-      <c r="E16" s="33"/>
-      <c r="F16" s="23"/>
+      <c r="D16" s="32">
+        <v>25</v>
+      </c>
+      <c r="E16" s="33" t="s">
+        <v>15</v>
+      </c>
+      <c r="F16" s="23" t="s">
+        <v>42</v>
+      </c>
       <c r="G16" s="39"/>
       <c r="O16">
         <v>40</v>
@@ -10955,11 +10977,11 @@
       </c>
       <c r="B7">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Plannification!E7,'Journal de travail'!$D$7:$D$532)</f>
-        <v>205</v>
+        <v>255</v>
       </c>
       <c r="C7">
         <f t="shared" si="0"/>
-        <v>265</v>
+        <v>315</v>
       </c>
       <c r="E7" s="73" t="str">
         <f>'Journal de travail'!M9</f>
@@ -10967,7 +10989,7 @@
       </c>
       <c r="F7" s="74" t="str">
         <f t="shared" ref="F7:F11" si="1">QUOTIENT(SUM(A7:B7),60)&amp;" h "&amp;TEXT(MOD(SUM(A7:B7),60), "00")&amp;" min"</f>
-        <v>4 h 25 min</v>
+        <v>5 h 15 min</v>
       </c>
       <c r="G7" s="75">
         <f t="shared" ref="G7:G9" si="2">SUM(A7:B7)/$C$11</f>
@@ -11101,22 +11123,22 @@
       </c>
       <c r="B11">
         <f>SUM(B6:B10)</f>
-        <v>205</v>
+        <v>255</v>
       </c>
       <c r="C11">
         <f>SUM(A11:B11)</f>
-        <v>265</v>
+        <v>315</v>
       </c>
       <c r="E11" s="81" t="s">
         <v>29</v>
       </c>
       <c r="F11" s="71" t="str">
         <f t="shared" si="1"/>
-        <v>4 h 25 min</v>
+        <v>5 h 15 min</v>
       </c>
       <c r="G11" s="82">
         <f>C11/C12</f>
-        <v>4.9074074074074076E-2</v>
+        <v>5.8333333333333334E-2</v>
       </c>
       <c r="L11" s="56" t="s">
         <v>29</v>

</xml_diff>